<commit_message>
change font to en "total"
</commit_message>
<xml_diff>
--- a/FMBrandFY2026FebRollingCost20260420.xlsx
+++ b/FMBrandFY2026FebRollingCost20260420.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHENKA~1\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F0BCD30-6EAE-4D4A-912E-434AFD7412E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D77B4316-1104-40B6-844A-D0F6755DA340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{43669CF1-3978-4373-A0CC-151DEED85F9B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{6D107D40-96C3-4FDD-8121-D26A6C0D666F}"/>
   </bookViews>
   <sheets>
     <sheet name="CostCenterGroupBySumResult" sheetId="1" r:id="rId1"/>
@@ -533,7 +533,7 @@
     <t>FY26 New Door</t>
   </si>
   <si>
-    <t>合计：</t>
+    <t>Total：</t>
   </si>
   <si>
     <t>KL</t>
@@ -555,7 +555,7 @@
     <t>KLFMFY2026000005</t>
   </si>
   <si>
-    <t>KL合计：</t>
+    <t>KL Total：</t>
   </si>
   <si>
     <t>Y</t>
@@ -577,7 +577,7 @@
     <t>KLFMFY2026000006</t>
   </si>
   <si>
-    <t>FM合计：</t>
+    <t>FM Total：</t>
   </si>
 </sst>
 </file>
@@ -1033,7 +1033,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D65DBDFD-4B9E-4EF4-8D22-D1A14E81C27D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83A6633D-0ACE-452A-82D8-6836BB785CC9}">
   <dimension ref="A1:DC33"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>